<commit_message>
#20 Altium BOM added @Ahsan96moten
</commit_message>
<xml_diff>
--- a/Design-Files/Tracker-pro-airbnb-v1.1/BOM/Altium_BOM_tracker-pro-airbnb-v1.1.xlsx
+++ b/Design-Files/Tracker-pro-airbnb-v1.1/BOM/Altium_BOM_tracker-pro-airbnb-v1.1.xlsx
@@ -5,21 +5,21 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ashan moten\Downloads\Tracker-pro-airbnb-v1.1\Tracker-pro-airbnb-v1.1\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="644">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="644">
   <si>
     <t>#</t>
   </si>
@@ -1956,8 +1956,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="13">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2046,6 +2046,14 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2258,7 +2266,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2316,15 +2324,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2333,9 +2332,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2346,6 +2342,12 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2654,10 +2656,10 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="2"/>
@@ -3785,12 +3787,12 @@
       <c r="L35" s="9"/>
     </row>
     <row r="36" spans="1:12" ht="36">
-      <c r="A36" s="28"/>
-      <c r="B36" s="29">
+      <c r="A36" s="24"/>
+      <c r="B36" s="25">
         <f t="shared" ref="B36" si="1">ROW(B36) - ROW($B$2)</f>
         <v>34</v>
       </c>
-      <c r="C36" s="30" t="s">
+      <c r="C36" s="26" t="s">
         <v>16</v>
       </c>
       <c r="D36" s="9" t="s">
@@ -3811,7 +3813,7 @@
       <c r="I36" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="J36" s="31"/>
+      <c r="J36" s="27"/>
       <c r="K36" s="17">
         <v>1</v>
       </c>
@@ -3859,29 +3861,31 @@
       <c r="C38" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="D38" s="28" t="s">
         <v>159</v>
       </c>
-      <c r="E38" s="10" t="s">
+      <c r="E38" s="28" t="s">
         <v>160</v>
       </c>
-      <c r="F38" s="9" t="s">
+      <c r="F38" s="28" t="s">
         <v>161</v>
       </c>
-      <c r="G38" s="10" t="s">
+      <c r="G38" s="28" t="s">
         <v>162</v>
       </c>
-      <c r="H38" s="9" t="s">
+      <c r="H38" s="28" t="s">
         <v>163</v>
       </c>
-      <c r="I38" s="10" t="s">
+      <c r="I38" s="28" t="s">
         <v>164</v>
       </c>
-      <c r="J38" s="16"/>
-      <c r="K38" s="17">
-        <v>1</v>
-      </c>
-      <c r="L38" s="9"/>
+      <c r="J38" s="28"/>
+      <c r="K38" s="28">
+        <v>1</v>
+      </c>
+      <c r="L38" s="20" t="s">
+        <v>308</v>
+      </c>
     </row>
     <row r="39" spans="1:12" ht="24">
       <c r="A39" s="2"/>
@@ -4312,7 +4316,7 @@
       </c>
       <c r="L51" s="12"/>
     </row>
-    <row r="52" spans="1:12">
+    <row r="52" spans="1:12" ht="24">
       <c r="A52" s="2"/>
       <c r="B52" s="7">
         <f>ROW(B52)-ROW($B$2)</f>
@@ -4847,26 +4851,26 @@
       <c r="C68" s="8" t="s">
         <v>302</v>
       </c>
-      <c r="D68" s="20" t="s">
+      <c r="D68" s="28" t="s">
         <v>303</v>
       </c>
-      <c r="E68" s="21" t="s">
+      <c r="E68" s="28" t="s">
         <v>304</v>
       </c>
-      <c r="F68" s="20" t="s">
+      <c r="F68" s="28" t="s">
         <v>305</v>
       </c>
-      <c r="G68" s="21" t="s">
+      <c r="G68" s="28" t="s">
         <v>306</v>
       </c>
-      <c r="H68" s="20" t="s">
+      <c r="H68" s="28" t="s">
         <v>307</v>
       </c>
-      <c r="I68" s="21" t="s">
+      <c r="I68" s="28" t="s">
         <v>164</v>
       </c>
-      <c r="J68" s="22"/>
-      <c r="K68" s="23">
+      <c r="J68" s="28"/>
+      <c r="K68" s="28">
         <v>1</v>
       </c>
       <c r="L68" s="20" t="s">
@@ -5377,29 +5381,31 @@
       <c r="C84" s="8" t="s">
         <v>330</v>
       </c>
-      <c r="D84" s="9" t="s">
+      <c r="D84" s="28" t="s">
         <v>369</v>
       </c>
-      <c r="E84" s="10" t="s">
+      <c r="E84" s="28" t="s">
         <v>370</v>
       </c>
-      <c r="F84" s="9" t="s">
+      <c r="F84" s="28" t="s">
         <v>333</v>
       </c>
-      <c r="G84" s="10" t="s">
+      <c r="G84" s="28" t="s">
         <v>371</v>
       </c>
-      <c r="H84" s="9" t="s">
+      <c r="H84" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="I84" s="10" t="s">
+      <c r="I84" s="28" t="s">
         <v>164</v>
       </c>
-      <c r="J84" s="16"/>
-      <c r="K84" s="17">
-        <v>1</v>
-      </c>
-      <c r="L84" s="9"/>
+      <c r="J84" s="28"/>
+      <c r="K84" s="28">
+        <v>1</v>
+      </c>
+      <c r="L84" s="20" t="s">
+        <v>308</v>
+      </c>
     </row>
     <row r="85" spans="1:12">
       <c r="A85" s="2"/>
@@ -7243,7 +7249,7 @@
       <c r="I140" s="10" t="s">
         <v>627</v>
       </c>
-      <c r="J140" s="24"/>
+      <c r="J140" s="21"/>
       <c r="K140" s="17">
         <v>1</v>
       </c>
@@ -7308,7 +7314,7 @@
       <c r="I142" s="13" t="s">
         <v>637</v>
       </c>
-      <c r="J142" s="25" t="s">
+      <c r="J142" s="22" t="s">
         <v>638</v>
       </c>
       <c r="K142" s="19">
@@ -7374,7 +7380,7 @@
       <c r="I144" s="13" t="s">
         <v>634</v>
       </c>
-      <c r="J144" s="26" t="s">
+      <c r="J144" s="23" t="s">
         <v>638</v>
       </c>
       <c r="K144" s="19">

</xml_diff>

<commit_message>
Battery Holder link added in BOM #20
</commit_message>
<xml_diff>
--- a/Design-Files/Tracker-pro-airbnb-v1.1/BOM/Altium_BOM_tracker-pro-airbnb-v1.1.xlsx
+++ b/Design-Files/Tracker-pro-airbnb-v1.1/BOM/Altium_BOM_tracker-pro-airbnb-v1.1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\ezlo-ambienttrackerpro-airbnb-hardware\Design-Files\Tracker-pro-airbnb-v1.1\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1006" uniqueCount="644">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="645">
   <si>
     <t>#</t>
   </si>
@@ -1951,12 +1951,15 @@
   </si>
   <si>
     <t>VKMD1451K101MV</t>
+  </si>
+  <si>
+    <t>Battery Holder</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="14">
     <font>
       <sz val="11"/>
@@ -2266,7 +2269,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2348,6 +2351,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2632,7 +2638,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L144"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="4.42578125" style="1" customWidth="1"/>
@@ -4316,7 +4322,7 @@
       </c>
       <c r="L51" s="12"/>
     </row>
-    <row r="52" spans="1:12" ht="24">
+    <row r="52" spans="1:12">
       <c r="A52" s="2"/>
       <c r="B52" s="7">
         <f>ROW(B52)-ROW($B$2)</f>
@@ -7354,9 +7360,9 @@
       </c>
       <c r="L143" s="12"/>
     </row>
-    <row r="144" spans="1:12">
+    <row r="144" spans="1:12" ht="15.75" thickBot="1">
       <c r="B144" s="7">
-        <f t="shared" ref="B144" si="2">ROW(B144)-ROW($B$2)</f>
+        <f t="shared" ref="B144:B145" si="2">ROW(B144)-ROW($B$2)</f>
         <v>142</v>
       </c>
       <c r="C144" s="11" t="s">
@@ -7387,6 +7393,40 @@
         <v>1</v>
       </c>
       <c r="L144" s="12"/>
+    </row>
+    <row r="145" spans="2:12" ht="15.75" thickBot="1">
+      <c r="B145" s="7">
+        <f t="shared" si="2"/>
+        <v>143</v>
+      </c>
+      <c r="C145" s="11" t="s">
+        <v>633</v>
+      </c>
+      <c r="D145" s="12" t="s">
+        <v>634</v>
+      </c>
+      <c r="E145" s="13" t="s">
+        <v>644</v>
+      </c>
+      <c r="F145" s="12" t="s">
+        <v>634</v>
+      </c>
+      <c r="G145" s="13" t="s">
+        <v>634</v>
+      </c>
+      <c r="H145" s="12" t="s">
+        <v>634</v>
+      </c>
+      <c r="I145" s="13" t="s">
+        <v>634</v>
+      </c>
+      <c r="J145" s="30" t="s">
+        <v>638</v>
+      </c>
+      <c r="K145" s="19">
+        <v>2</v>
+      </c>
+      <c r="L145" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -7395,6 +7435,7 @@
   <hyperlinks>
     <hyperlink ref="J142" r:id="rId1"/>
     <hyperlink ref="J144" r:id="rId2"/>
+    <hyperlink ref="J145" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
#20 Battery added in Altium BOM .
</commit_message>
<xml_diff>
--- a/Design-Files/Tracker-pro-airbnb-v1.1/BOM/Altium_BOM_tracker-pro-airbnb-v1.1.xlsx
+++ b/Design-Files/Tracker-pro-airbnb-v1.1/BOM/Altium_BOM_tracker-pro-airbnb-v1.1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\ezlo-ambienttrackerpro-airbnb-hardware\Design-Files\Tracker-pro-airbnb-v1.1\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ezlo-ambienttrackerpro-airbnb-hardware\Design-Files\Tracker-pro-airbnb-v1.1\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="645">
   <si>
     <t>#</t>
   </si>
@@ -1959,7 +1959,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="14">
     <font>
       <sz val="11"/>
@@ -1972,14 +1972,14 @@
       <sz val="10"/>
       <color indexed="13"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1987,27 +1987,27 @@
       <sz val="10"/>
       <color theme="0"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2015,7 +2015,7 @@
       <sz val="11"/>
       <color rgb="FF800080"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2023,7 +2023,7 @@
       <sz val="11"/>
       <color theme="10"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2349,11 +2349,11 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2638,7 +2638,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L145"/>
+  <dimension ref="A1:L146"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="4.42578125" style="1" customWidth="1"/>
@@ -2662,10 +2662,10 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="2"/>
@@ -7362,7 +7362,7 @@
     </row>
     <row r="144" spans="1:12" ht="15.75" thickBot="1">
       <c r="B144" s="7">
-        <f t="shared" ref="B144:B145" si="2">ROW(B144)-ROW($B$2)</f>
+        <f t="shared" ref="B144:B146" si="2">ROW(B144)-ROW($B$2)</f>
         <v>142</v>
       </c>
       <c r="C144" s="11" t="s">
@@ -7420,13 +7420,47 @@
       <c r="I145" s="13" t="s">
         <v>634</v>
       </c>
-      <c r="J145" s="30" t="s">
+      <c r="J145" s="29" t="s">
         <v>638</v>
       </c>
       <c r="K145" s="19">
         <v>2</v>
       </c>
       <c r="L145" s="12"/>
+    </row>
+    <row r="146" spans="2:12" ht="15.75" thickBot="1">
+      <c r="B146" s="7">
+        <f t="shared" si="2"/>
+        <v>144</v>
+      </c>
+      <c r="C146" s="11" t="s">
+        <v>633</v>
+      </c>
+      <c r="D146" s="12" t="s">
+        <v>634</v>
+      </c>
+      <c r="E146" s="13" t="s">
+        <v>636</v>
+      </c>
+      <c r="F146" s="12" t="s">
+        <v>634</v>
+      </c>
+      <c r="G146" s="13" t="s">
+        <v>634</v>
+      </c>
+      <c r="H146" s="12" t="s">
+        <v>634</v>
+      </c>
+      <c r="I146" s="13" t="s">
+        <v>634</v>
+      </c>
+      <c r="J146" s="29" t="s">
+        <v>638</v>
+      </c>
+      <c r="K146" s="19">
+        <v>2</v>
+      </c>
+      <c r="L146" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -7436,6 +7470,7 @@
     <hyperlink ref="J142" r:id="rId1"/>
     <hyperlink ref="J144" r:id="rId2"/>
     <hyperlink ref="J145" r:id="rId3"/>
+    <hyperlink ref="J146" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
#20 Battery Update in BOM
</commit_message>
<xml_diff>
--- a/Design-Files/Tracker-pro-airbnb-v1.1/BOM/Altium_BOM_tracker-pro-airbnb-v1.1.xlsx
+++ b/Design-Files/Tracker-pro-airbnb-v1.1/BOM/Altium_BOM_tracker-pro-airbnb-v1.1.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1022" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="645">
   <si>
     <t>#</t>
   </si>
@@ -1926,15 +1926,9 @@
     <t>-</t>
   </si>
   <si>
-    <t>3.7V 3000mAh 505080 Polymer Lithium Lipo Rechargeable battery for GPS DVD PAD power bank e-book camera tablet 5*50*80mm</t>
-  </si>
-  <si>
     <t>Battery</t>
   </si>
   <si>
-    <t>3000mAh</t>
-  </si>
-  <si>
     <t>Aliexpress</t>
   </si>
   <si>
@@ -1954,6 +1948,12 @@
   </si>
   <si>
     <t>Battery Holder</t>
+  </si>
+  <si>
+    <t>1-2PCS 3.7V 1000mAh 10440 ICR10440 3A Lithium Rechargeable Battery For Flashlight Camera Shaver Power Torch Remote Li-ion Cell</t>
+  </si>
+  <si>
+    <t>3.7V</t>
   </si>
 </sst>
 </file>
@@ -2269,7 +2269,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2328,9 +2328,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2638,7 +2635,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L146"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="4.42578125" style="1" customWidth="1"/>
@@ -2662,10 +2659,10 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="2"/>
@@ -3793,25 +3790,25 @@
       <c r="L35" s="9"/>
     </row>
     <row r="36" spans="1:12" ht="36">
-      <c r="A36" s="24"/>
-      <c r="B36" s="25">
+      <c r="A36" s="23"/>
+      <c r="B36" s="24">
         <f t="shared" ref="B36" si="1">ROW(B36) - ROW($B$2)</f>
         <v>34</v>
       </c>
-      <c r="C36" s="26" t="s">
+      <c r="C36" s="25" t="s">
         <v>16</v>
       </c>
       <c r="D36" s="9" t="s">
         <v>152</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="H36" s="9" t="s">
         <v>107</v>
@@ -3819,7 +3816,7 @@
       <c r="I36" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="J36" s="27"/>
+      <c r="J36" s="26"/>
       <c r="K36" s="17">
         <v>1</v>
       </c>
@@ -3867,26 +3864,26 @@
       <c r="C38" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="D38" s="28" t="s">
+      <c r="D38" s="27" t="s">
         <v>159</v>
       </c>
-      <c r="E38" s="28" t="s">
+      <c r="E38" s="27" t="s">
         <v>160</v>
       </c>
-      <c r="F38" s="28" t="s">
+      <c r="F38" s="27" t="s">
         <v>161</v>
       </c>
-      <c r="G38" s="28" t="s">
+      <c r="G38" s="27" t="s">
         <v>162</v>
       </c>
-      <c r="H38" s="28" t="s">
+      <c r="H38" s="27" t="s">
         <v>163</v>
       </c>
-      <c r="I38" s="28" t="s">
+      <c r="I38" s="27" t="s">
         <v>164</v>
       </c>
-      <c r="J38" s="28"/>
-      <c r="K38" s="28">
+      <c r="J38" s="27"/>
+      <c r="K38" s="27">
         <v>1</v>
       </c>
       <c r="L38" s="20" t="s">
@@ -4857,26 +4854,26 @@
       <c r="C68" s="8" t="s">
         <v>302</v>
       </c>
-      <c r="D68" s="28" t="s">
+      <c r="D68" s="27" t="s">
         <v>303</v>
       </c>
-      <c r="E68" s="28" t="s">
+      <c r="E68" s="27" t="s">
         <v>304</v>
       </c>
-      <c r="F68" s="28" t="s">
+      <c r="F68" s="27" t="s">
         <v>305</v>
       </c>
-      <c r="G68" s="28" t="s">
+      <c r="G68" s="27" t="s">
         <v>306</v>
       </c>
-      <c r="H68" s="28" t="s">
+      <c r="H68" s="27" t="s">
         <v>307</v>
       </c>
-      <c r="I68" s="28" t="s">
+      <c r="I68" s="27" t="s">
         <v>164</v>
       </c>
-      <c r="J68" s="28"/>
-      <c r="K68" s="28">
+      <c r="J68" s="27"/>
+      <c r="K68" s="27">
         <v>1</v>
       </c>
       <c r="L68" s="20" t="s">
@@ -5387,26 +5384,26 @@
       <c r="C84" s="8" t="s">
         <v>330</v>
       </c>
-      <c r="D84" s="28" t="s">
+      <c r="D84" s="27" t="s">
         <v>369</v>
       </c>
-      <c r="E84" s="28" t="s">
+      <c r="E84" s="27" t="s">
         <v>370</v>
       </c>
-      <c r="F84" s="28" t="s">
+      <c r="F84" s="27" t="s">
         <v>333</v>
       </c>
-      <c r="G84" s="28" t="s">
+      <c r="G84" s="27" t="s">
         <v>371</v>
       </c>
-      <c r="H84" s="28" t="s">
+      <c r="H84" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="I84" s="28" t="s">
+      <c r="I84" s="27" t="s">
         <v>164</v>
       </c>
-      <c r="J84" s="28"/>
-      <c r="K84" s="28">
+      <c r="J84" s="27"/>
+      <c r="K84" s="27">
         <v>1</v>
       </c>
       <c r="L84" s="20" t="s">
@@ -7261,7 +7258,7 @@
       </c>
       <c r="L140" s="9"/>
     </row>
-    <row r="141" spans="1:12">
+    <row r="141" spans="1:12" ht="15.75" thickBot="1">
       <c r="A141" s="2"/>
       <c r="B141" s="7">
         <f t="shared" si="0"/>
@@ -7294,7 +7291,7 @@
       </c>
       <c r="L141" s="12"/>
     </row>
-    <row r="142" spans="1:12" ht="48">
+    <row r="142" spans="1:12" ht="48.75" thickBot="1">
       <c r="B142" s="7">
         <f t="shared" si="0"/>
         <v>140</v>
@@ -7306,29 +7303,29 @@
         <v>634</v>
       </c>
       <c r="E142" s="13" t="s">
-        <v>635</v>
+        <v>643</v>
       </c>
       <c r="F142" s="12" t="s">
         <v>634</v>
       </c>
       <c r="G142" s="13" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="H142" s="12" t="s">
         <v>634</v>
       </c>
       <c r="I142" s="13" t="s">
-        <v>637</v>
-      </c>
-      <c r="J142" s="22" t="s">
-        <v>638</v>
+        <v>644</v>
+      </c>
+      <c r="J142" s="28" t="s">
+        <v>636</v>
       </c>
       <c r="K142" s="19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L142" s="12"/>
     </row>
-    <row r="143" spans="1:12">
+    <row r="143" spans="1:12" ht="15.75" thickBot="1">
       <c r="B143" s="7">
         <f t="shared" si="0"/>
         <v>141</v>
@@ -7340,13 +7337,13 @@
         <v>634</v>
       </c>
       <c r="E143" s="13" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="F143" s="12" t="s">
         <v>634</v>
       </c>
       <c r="G143" s="13" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="H143" s="12" t="s">
         <v>634</v>
@@ -7362,7 +7359,7 @@
     </row>
     <row r="144" spans="1:12" ht="15.75" thickBot="1">
       <c r="B144" s="7">
-        <f t="shared" ref="B144:B146" si="2">ROW(B144)-ROW($B$2)</f>
+        <f t="shared" ref="B144:B145" si="2">ROW(B144)-ROW($B$2)</f>
         <v>142</v>
       </c>
       <c r="C144" s="11" t="s">
@@ -7372,13 +7369,13 @@
         <v>634</v>
       </c>
       <c r="E144" s="13" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="F144" s="12" t="s">
         <v>634</v>
       </c>
       <c r="G144" s="13" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="H144" s="12" t="s">
         <v>634</v>
@@ -7386,8 +7383,8 @@
       <c r="I144" s="13" t="s">
         <v>634</v>
       </c>
-      <c r="J144" s="23" t="s">
-        <v>638</v>
+      <c r="J144" s="22" t="s">
+        <v>636</v>
       </c>
       <c r="K144" s="19">
         <v>1</v>
@@ -7406,7 +7403,7 @@
         <v>634</v>
       </c>
       <c r="E145" s="13" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="F145" s="12" t="s">
         <v>634</v>
@@ -7420,57 +7417,22 @@
       <c r="I145" s="13" t="s">
         <v>634</v>
       </c>
-      <c r="J145" s="29" t="s">
-        <v>638</v>
+      <c r="J145" s="28" t="s">
+        <v>636</v>
       </c>
       <c r="K145" s="19">
         <v>2</v>
       </c>
       <c r="L145" s="12"/>
-    </row>
-    <row r="146" spans="2:12" ht="15.75" thickBot="1">
-      <c r="B146" s="7">
-        <f t="shared" si="2"/>
-        <v>144</v>
-      </c>
-      <c r="C146" s="11" t="s">
-        <v>633</v>
-      </c>
-      <c r="D146" s="12" t="s">
-        <v>634</v>
-      </c>
-      <c r="E146" s="13" t="s">
-        <v>636</v>
-      </c>
-      <c r="F146" s="12" t="s">
-        <v>634</v>
-      </c>
-      <c r="G146" s="13" t="s">
-        <v>634</v>
-      </c>
-      <c r="H146" s="12" t="s">
-        <v>634</v>
-      </c>
-      <c r="I146" s="13" t="s">
-        <v>634</v>
-      </c>
-      <c r="J146" s="29" t="s">
-        <v>638</v>
-      </c>
-      <c r="K146" s="19">
-        <v>2</v>
-      </c>
-      <c r="L146" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="I1:L1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="J142" r:id="rId1"/>
-    <hyperlink ref="J144" r:id="rId2"/>
-    <hyperlink ref="J145" r:id="rId3"/>
-    <hyperlink ref="J146" r:id="rId4"/>
+    <hyperlink ref="J144" r:id="rId1"/>
+    <hyperlink ref="J145" r:id="rId2"/>
+    <hyperlink ref="J142" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>